<commit_message>
Remove requirement text from the exercise workbooks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HiyVPr15dFfxwtDW3Tiv76
</commit_message>
<xml_diff>
--- a/excel_bai_tap/bai1_diem_thi_nghe.xlsx
+++ b/excel_bai_tap/bai1_diem_thi_nghe.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">ĐIỂM THI NGHỀ NĂM HỌC 2017 - 2018</t>
   </si>
@@ -77,39 +77,6 @@
   </si>
   <si>
     <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yêu cầu:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Điểm Word + Excel: điểm word là kí tự 1,2 của điểm; điểm excel là kí tự 3,4 của điểm và tính trung bình</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Điểm thực hành: là kí tự 5,6 của điểm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Điểm TB: (điểm word excel + điểm th*3)/4 làm tròn đến 2 số thập phân</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Kết quả: nếu điểm tb&gt;=5 thì "đậu"; nếu điểm tb&lt;5 thì "rớt"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Xếp loại:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nếu điểm tb&gt;=8 thì "giỏi"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nếu điểm tb&gt;=6.5 thì "khá"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nếu điểm tb&gt;=5 thì "tb"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nếu điểm tb&lt;5 thì "yếu - kém"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Học bổng: nếu đối tượng là A hoặc B và điểm tb&gt;=8.0 thì học bổng là 5000000</t>
   </si>
 </sst>
 </file>
@@ -124,7 +91,7 @@
     <numFmt numFmtId="168" formatCode="0.00"/>
     <numFmt numFmtId="169" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,14 +132,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="0"/>
@@ -228,7 +187,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -266,14 +225,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -469,7 +420,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -624,61 +575,6 @@
       <c r="I5" s="9" t="n">
         <f aca="false">IF(AND(OR(C5="A",C5="B"),F5&gt;=8),5000000,0)</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>